<commit_message>
SPM-33: make the Readiness tab clearer for a first-time user
The state badges moved between the top-right and below the text depending
on whether a row had a button, and each row showed two unlabelled badges
(e.g. "Approved" beside "Complete").

- Items are grouped into Venue bookings, Equipment, Registration and
  Safety check; an empty section says so.
- Every row has the same three columns: where it stands first, then what
  it is, then the action.
- An item's own status is labelled ("Booking status: Pending",
  "Request status: Reserved"), so it is not read as whether it is done.
- A key under the summary says what Complete, Outstanding and Not
  required mean.
- A confirmed event says "This event is confirmed" instead of the
  blocking count.

Six page tests added; manual cases TC02 and TC15 updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-33_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-33_Test_Cases.xlsx
@@ -2729,7 +2729,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="98.5" customHeight="1">
+    <row r="7" ht="112" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2738,7 +2738,7 @@
       <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 2: The event opens with the status badge 'Confirmed'.
-Step 3: 'Orchard Gallery' shows 'Complete'. 'Portable Stage' shows 'Not required' and 'Cannot be provided', and says 'Marked as not required by Daniel Tan on 1 Oct 2026, 10:00'. There is no 'Mark as required' or 'Mark as not required' button on any item: arrangements are marked only while the event is in Planning.</t>
+Step 3: The message 'This event is confirmed' is shown in place of the count of blocking arrangements. 'Orchard Gallery' shows 'Complete'. 'Portable Stage' shows 'Not required' and 'Cannot be provided', and says 'Marked as not required by Daniel Tan on 1 Oct 2026, 10:00'. There is no 'Mark as required' or 'Mark as not required' button on any item: arrangements are marked only while the event is in Planning.</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3361,6 +3361,17 @@
         </is>
       </c>
       <c r="C16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="179.5" customHeight="1">
+      <c r="A17" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-12, layout (cleaned up for a first-time user): the Readiness tab groups its items into 'Venue bookings', 'Equipment', 'Registration' and 'Safety check' sections. Every item shows where it stands ('Complete', 'Outstanding' or 'Not required') first, in the same place, then its name, then the action. Its own status is written out with what it is the status of - 'Booking status: Pending', 'Request status: Reserved', 'Safety check status: Awaiting review' - so it is not mistaken for whether it is done. A key under the summary says what the three states mean: 'In place.', 'Still to be done.', 'Marked as not needed for this event.' An empty section says 'No equipment has been recorded for this event.' or 'Registration is not enabled for this event.' A confirmed event shows 'This event is confirmed' instead of the blocking count, and its subtitle reads 'What this event was confirmed with.'</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3632,7 +3643,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="85" customHeight="1">
+    <row r="7" ht="112" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3640,7 +3651,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 3: Apart from the 'Operational Safety Check' (Not submitted), the list has one item, 'No venue booked', showing 'Outstanding' and saying no venue is booked for this event. It has no 'Mark as not required' button. No equipment item and no 'Registration setup' item is listed. The message '1 arrangement still blocks confirmation' is shown.</t>
+          <t>Step 3: Apart from the 'Operational Safety Check' (Not submitted), the list has one item, 'No venue booked', showing 'Outstanding' and saying no venue is booked for this event. It has no 'Mark as not required' button. The Equipment section says 'No equipment has been recorded for this event.' and the Registration section says 'Registration is not enabled for this event.' The message '1 arrangement still blocks confirmation' is shown.</t>
         </is>
       </c>
     </row>

</xml_diff>